<commit_message>
docs(plan): finalize 4-member task assignment and progress reports without Tran Van Nhat, independent roles with deep business logic
</commit_message>
<xml_diff>
--- a/BAO_CAO_TIEN_DO_TUAN_3_FA26SE032.xlsx
+++ b/BAO_CAO_TIEN_DO_TUAN_3_FA26SE032.xlsx
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1493,64 +1493,6 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Trần Văn Nhật</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>nhat</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>FR-07, FR-08</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>Media Hub kho nội dung quảng bá &amp; Liên kết tài khoản mạng xã hội KOL</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>frontend/src/pages/collaborator/MarketingToolkitPage.tsx
-frontend/src/pages/collaborator/SocialChannelsPage.tsx</t>
-        </is>
-      </c>
-      <c r="G12" s="19" t="inlineStr">
-        <is>
-          <t>GET /api/v1/media-hub
-POST /api/v1/social-channels/link</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>backend/src/modules/media/media.service.ts
-backend/src/modules/social-channels/</t>
-        </is>
-      </c>
-      <c r="I12" s="19" t="inlineStr">
-        <is>
-          <t>media_assets, social_accounts</t>
-        </is>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>COMPLETED 100%</t>
-        </is>
-      </c>
-      <c r="K12" s="18" t="inlineStr">
-        <is>
-          <t>PR #42, #43</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1562,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1675,7 +1617,7 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>2. DANH SÁCH SINH VIÊN THỰC HIỆN ĐỒ ÁN</t>
+          <t>2. DANH SÁCH SINH VIÊN THỰC HIỆN ĐỒ ÁN (NHÓM 4 THÀNH VIÊN CHÍNH THỨC)</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1689,7 @@
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>Kiến trúc tổng thể, Core IAM đa vai trò, Phân quyền RBAC, Quản lý Gian hàng &amp; Sản phẩm, Escrow 14 ngày &amp; Tích hợp sàn (FR-01 → FR-08, FR-17 → FR-20).</t>
+          <t>Kiến trúc hệ thống, Core IAM đa vai trò, Bảo mật Argon2id/JWT/OTP, Cơ chế Escrow 14 ngày, Cổng trọng tài phân xử tranh chấp &amp; Thiết kế Design System Vàng Be.</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1724,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Động cơ Tracking Smart Link &amp; Dynamic QR Code, Last-Click Cookie 30 ngày, Redis Rate Limit chống spam click, UI Marketplace &amp; Search Zoom (FR-09 → FR-16).</t>
+          <t>Tiếp thị liên kết KOL/KOC, Phân cấp hoa hồng 2 tầng (Open vs Exclusive), Quy trình cấp hàng mẫu 4 bước, Voucher phiên Livestream &amp; Phê duyệt Shop Onboarding (KYC) / Sản phẩm.</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1759,7 @@
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
-          <t>Động cơ AI Fraud Sentinel phát hiện gian lận traffic, Hệ thống Audit Logs an ninh bất biến, Trợ lý AI gợi ý KOL phù hợp (FR-30, FR-31, FR-32).</t>
+          <t>Phân hệ Chủ Gian Hàng (Merchant Operations), Quản lý tồn kho real-time &amp; cảnh báo tồn &lt;= 5, Shop chủ động hủy đơn &amp; hoàn tiền, Bộ mô phỏng vận chuyển Shipping Simulator in phiếu A6 barcode, Tiếp nhận đổi trả phía Shop.</t>
         </is>
       </c>
     </row>
@@ -1852,42 +1794,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Ví điện tử CTV, Đối soát hoa hồng tự động, Quy trình Batch Payout xuất file VietQR Napas247 XLSX và Khấu trừ thuế TNCN 10% (FR-21 → FR-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Trần Văn Nhật</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>SE172768</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>0949997692</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>NhatTVSE172768@fpt.efu.vn</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>Thành viên (Member)</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>Kho nội dung số tập trung Media Hub, Quản lý liên kết mạng xã hội KOL, Hệ thống Chat trao đổi KOL - Shop qua Socket.io realtime (FR-07, FR-08, FR-26).</t>
+          <t>Cổng Khách Hàng (Customer Portal), Giỏ hàng đồng bộ Database PostgreSQL, Quy trình gửi yêu cầu Đổi trả 14 ngày kèm video mở hộp, Ràng buộc đánh giá thật Review Gate (đơn COMPLETED), Kênh chat tư vấn Khách ⇄ Shop.</t>
         </is>
       </c>
     </row>

</xml_diff>